<commit_message>
feat: apply revised ego-ok 90 personality items to 99-item source bank
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/docs/internal-materials/ego-ok/items-99-excel-export.xlsx
+++ b/docs/internal-materials/ego-ok/items-99-excel-export.xlsx
@@ -428,7 +428,7 @@
         <v>1</v>
       </c>
       <c r="B2" t="str">
-        <v>다른 사람의 부족한 점보다는 장점을 먼저 찾아, 따뜻하게 칭찬하고 격려하는 편이다.</v>
+        <v>다른 사람의 단점을 지적하기보다, 장점을 찾아 자연스럽게 칭찬하곤 한다.</v>
       </c>
       <c r="C2" t="str">
         <v>np_positive</v>
@@ -445,7 +445,7 @@
         <v>2</v>
       </c>
       <c r="B3" t="str">
-        <v>매사에 표정이나 감정 변화가 적어서, 사람들에게 딱딱하고 재미없다는 인상을 주는 편이다.</v>
+        <v>감정 변화가 적어서 주변에서, 차분하거나 무심해 보인다는 말을 듣곤 한다.</v>
       </c>
       <c r="C3" t="str">
         <v>a_negative</v>
@@ -462,7 +462,7 @@
         <v>3</v>
       </c>
       <c r="B4" t="str">
-        <v>부족한 면이 있더라도, 나 자신을 있는 그대로 아끼고 긍정적으로 바라본다.</v>
+        <v>대체로 나 자신을 긍정적으로 바라보는 편이다.</v>
       </c>
       <c r="C4" t="str">
         <v>i_plus</v>
@@ -479,7 +479,7 @@
         <v>4</v>
       </c>
       <c r="B5" t="str">
-        <v>일을 할 때 다른 사람들의 의견보다는, 내 방식대로 밀어붙이는 편이다.</v>
+        <v>일이나 모임을 주도할 때, 다른 사람의 의견보다 내 방식대로 밀어붙이곤 한다.</v>
       </c>
       <c r="C5" t="str">
         <v>cp_negative</v>
@@ -496,7 +496,7 @@
         <v>5</v>
       </c>
       <c r="B6" t="str">
-        <v>의견이나 살아온 방식이 나와 달라도, ‘틀렸다’고 단정하지 않고 있는 그대로 인정하는 편이다.</v>
+        <v>나와 생각이나 방식이 달라도, 대체로 인정하고 받아들이는 편이다.</v>
       </c>
       <c r="C6" t="str">
         <v>u_plus</v>
@@ -513,7 +513,7 @@
         <v>6</v>
       </c>
       <c r="B7" t="str">
-        <v>다른 사람들의 시선을 지나치게 의식해서, 대체로 행동이 조심스럽고 위축되는 편이다.</v>
+        <v>주변의 시선이나 평가를 의식하며, 스스로 편하게 행동하지 못하고 위축되곤 한다.</v>
       </c>
       <c r="C7" t="str">
         <v>ac_negative</v>
@@ -530,7 +530,7 @@
         <v>7</v>
       </c>
       <c r="B8" t="str">
-        <v>일상 속에서도, 때로는 아이처럼 순수하고 천진난만한 모습을 드러내곤 한다.</v>
+        <v>때로는 아이처럼 계산 없이, 순수한 마음으로 사람이나 상황을 대하곤 한다.</v>
       </c>
       <c r="C8" t="str">
         <v>fc_positive</v>
@@ -547,7 +547,7 @@
         <v>8</v>
       </c>
       <c r="B9" t="str">
-        <v>스스로 매력이 부족해서, 다른 사람들에게 별로 호감을 주지 못한다고 느낄 때가 많다.</v>
+        <v>다른 사람들에게 별로 호감을 주지 못한다고, 느낄 때가 많다.</v>
       </c>
       <c r="C9" t="str">
         <v>i_minus</v>
@@ -581,7 +581,7 @@
         <v>10</v>
       </c>
       <c r="B11" t="str">
-        <v>다른 사람을 평가할 때, 대체로 엄격하고 까다로운 기준을 두는 편이다.</v>
+        <v>다른 사람을 평가할 때, 엄격한 기준을 대는 편이다.</v>
       </c>
       <c r="C11" t="str">
         <v>u_minus</v>
@@ -598,7 +598,7 @@
         <v>11</v>
       </c>
       <c r="B12" t="str">
-        <v>어떤 상황에서도, 말과 행동이 차분하며 침착하게 이성을 유지하는 편이다.</v>
+        <v>갑작스럽거나 혼란스러운 상황이 생겨도, 당황하지 않고 차분히 대처하곤 한다.</v>
       </c>
       <c r="C12" t="str">
         <v>a_positive</v>
@@ -615,7 +615,7 @@
         <v>12</v>
       </c>
       <c r="B13" t="str">
-        <v>가족이나 주변 사람들의 작은 일까지도, 나도 모르게 끼어들어 간섭하는 경향이 있다.</v>
+        <v>가족이나 주변 사람들의 작은 일까지도, 나도 모르게 다가가 이것저것 챙기곤 한다.</v>
       </c>
       <c r="C13" t="str">
         <v>np_negative</v>
@@ -632,7 +632,7 @@
         <v>13</v>
       </c>
       <c r="B14" t="str">
-        <v>나는 내 주위와 사회에 나름대로 보탬이 되는, 가치 있는 사람이라고 생각한다.</v>
+        <v>주변이나 사회에서, 나름대로 도움이 되는 사람이라고 생각한다.</v>
       </c>
       <c r="C14" t="str">
         <v>i_plus</v>
@@ -649,7 +649,7 @@
         <v>14</v>
       </c>
       <c r="B15" t="str">
-        <v>상대방의 사소한 잘못이나 실수를 그냥 넘기지 않고, 분명하게 지적하는 편이다.</v>
+        <v>주변 사람들의 작은 실수나, 원칙에 어긋나는 행동을 그냥 지나치지 못하곤 한다.</v>
       </c>
       <c r="C15" t="str">
         <v>cp_negative</v>
@@ -683,7 +683,7 @@
         <v>16</v>
       </c>
       <c r="B17" t="str">
-        <v>다른 사람들과 의견 차이가 생기면, 원만하게 타협하고 맞춰가려고 노력하는 편이다.</v>
+        <v>다른 사람과 의견이 다를 때 고집을 부리기보다, 서로 양보하며 원만히 해결하곤 한다.</v>
       </c>
       <c r="C17" t="str">
         <v>ac_positive</v>
@@ -700,7 +700,7 @@
         <v>17</v>
       </c>
       <c r="B18" t="str">
-        <v>차분하고 깊게 생각하기보다, 그 순간의 감정과 기분에 이끌려 행동하는 편이다.</v>
+        <v>순간적인 기분이나 감정에 이끌려, 즉흥적으로 행동하곤 한다.</v>
       </c>
       <c r="C18" t="str">
         <v>fc_negative</v>
@@ -717,7 +717,7 @@
         <v>18</v>
       </c>
       <c r="B19" t="str">
-        <v>처음 만나는 사람이라도 거리를 두기보다, 먼저 열린 마음으로 친절하게 다가가는 편이다.</v>
+        <v>다른 사람이 자기주장을 당당하게 표현하는 것은, 물론이며 바람직하다고 본다.</v>
       </c>
       <c r="C19" t="str">
         <v>u_plus</v>
@@ -734,7 +734,7 @@
         <v>19</v>
       </c>
       <c r="B20" t="str">
-        <v>주변 사람들로부터 충분한 관심이나 지지를 받지 못해, 마음 한구석이 늘 허전한 편이다.</v>
+        <v>어릴 적부터 가족이나 주변에서, 환영받거나 사랑받지 못했다고 생각한다.</v>
       </c>
       <c r="C20" t="str">
         <v>i_minus</v>
@@ -751,7 +751,7 @@
         <v>20</v>
       </c>
       <c r="B21" t="str">
-        <v>다른 사람의 장점이나 좋은 성과를 앞에 두고도, 인정이나 칭찬을 하는 것이 쉽지 않은 편이다.</v>
+        <v>다른 사람의 장점을 보아도, 선뜻 칭찬해 주기는 망설이는 편이다.</v>
       </c>
       <c r="C21" t="str">
         <v>u_minus</v>
@@ -768,7 +768,7 @@
         <v>21</v>
       </c>
       <c r="B22" t="str">
-        <v>평소 다른 사람의 입장이나 사정을 먼저 챙기며, 따뜻하게 배려해 주는 편이다.</v>
+        <v>상대방의 이야기를 주의 깊게 들으며, 그 감정에 진심으로 공감해 주곤 한다.</v>
       </c>
       <c r="C22" t="str">
         <v>np_positive</v>
@@ -785,7 +785,7 @@
         <v>22</v>
       </c>
       <c r="B23" t="str">
-        <v>상대방의 마음에 공감해주기보다 사실과 논리만 따지다 보니, 대화가 대체로 차가워질 때가 많다.</v>
+        <v>대화할 때 상대의 기분이나 감정보다는, 담담하게 사실과 정보만 전달하곤 한다.</v>
       </c>
       <c r="C23" t="str">
         <v>a_negative</v>
@@ -802,7 +802,7 @@
         <v>23</v>
       </c>
       <c r="B24" t="str">
-        <v>다소 손해를 보거나 유혹이 있더라도, 양심과 도덕적 기준에 따라 행동하는 편이다.</v>
+        <v>현재에 머무르지 않고, 정해둔 목표를 향해 꾸준히 노력하곤 한다.</v>
       </c>
       <c r="C24" t="str">
         <v>cp_positive</v>
@@ -819,7 +819,7 @@
         <v>24</v>
       </c>
       <c r="B25" t="str">
-        <v>어려운 일들은 스스로 해결하기보다, 주변 사람에게 의지하거나 도움을 받으려는 경향이 있다.</v>
+        <v>판단하기 어려운 상황이 오면, 스스로 결정하기보다 남에게 의지하고 맡겨버리곤 한다.</v>
       </c>
       <c r="C25" t="str">
         <v>ac_negative</v>
@@ -836,7 +836,7 @@
         <v>25</v>
       </c>
       <c r="B26" t="str">
-        <v>나를 아는 사람들에게 나름대로 좋은 평가와 신뢰를 받고 있다고 여긴다.</v>
+        <v>주변에서는 대체로 좋은 신뢰와 인정을 받고 있다고 생각한다.</v>
       </c>
       <c r="C26" t="str">
         <v>i_plus</v>
@@ -870,7 +870,7 @@
         <v>27</v>
       </c>
       <c r="B28" t="str">
-        <v>주변 사람에게 좋은 일이나 성과가 생기면, 진심으로 기뻐하고 축하해 주는 편이다.</v>
+        <v>주변 사람이 잘되는 모습을 보면, 내 일처럼 기분이 좋아진다.</v>
       </c>
       <c r="C28" t="str">
         <v>u_plus</v>
@@ -887,7 +887,7 @@
         <v>28</v>
       </c>
       <c r="B29" t="str">
-        <v>남들의 시선이나 입장은 아랑곳하지 않고, 내가 하고 싶은 대로 행동하는 편이다.</v>
+        <v>주변 시선이나 규칙보다는, 내 기분이나 마음에 따라 내키는 대로 행동하곤 한다.</v>
       </c>
       <c r="C29" t="str">
         <v>fc_negative</v>
@@ -904,7 +904,7 @@
         <v>29</v>
       </c>
       <c r="B30" t="str">
-        <v>스스로의 능력이나 판단에 확신을 갖지 못하고, 늘 나 자신을 의심하는 편이다.</v>
+        <v>내 판단이나 능력에 확신이 서지 않아, 중요한 순간에 스스로를 의심하는 편이다.</v>
       </c>
       <c r="C30" t="str">
         <v>i_minus</v>
@@ -921,7 +921,7 @@
         <v>30</v>
       </c>
       <c r="B31" t="str">
-        <v>누군가 어려운 처지에 놓여도, 대개 본인이 자초한 결과라고 생각하는 편이다.</v>
+        <v>남이 어려움을 겪으면, 본인이 주의하지 않아서 생긴 일이라 생각하는 편이다.</v>
       </c>
       <c r="C31" t="str">
         <v>u_minus</v>
@@ -938,7 +938,7 @@
         <v>31</v>
       </c>
       <c r="B32" t="str">
-        <v>문제가 생겼을 때 개인적인 감정이나 기분에 치우치지 않고, 명확한 사실과 근거를 바탕으로 판단하는 편이다.</v>
+        <v>어떤 문제를 다룰 때 한쪽에 쏠리지 않고, 객관적인 사실에 근거해 판단하는 편이다.</v>
       </c>
       <c r="C32" t="str">
         <v>a_positive</v>
@@ -955,7 +955,7 @@
         <v>32</v>
       </c>
       <c r="B33" t="str">
-        <v>상대방이 알아서 할 수 있는 일인데도, 나도 모르게 사소한 것까지 일일이 다 챙겨주는 편이다.</v>
+        <v>일터에서 남의 역할까지, 나서서 맡아 하곤 한다.</v>
       </c>
       <c r="C33" t="str">
         <v>np_negative</v>
@@ -972,7 +972,7 @@
         <v>33</v>
       </c>
       <c r="B34" t="str">
-        <v>새로운 것을 배우고 경험하는 일에 호기심이 많고, 의욕과 열정이 넘치는 편이다.</v>
+        <v>새로운 분야나 낯선 경험을 접하면, 대체로 호기심을 가지고 즐겁게 시작한다.</v>
       </c>
       <c r="C34" t="str">
         <v>fc_positive</v>
@@ -989,7 +989,7 @@
         <v>34</v>
       </c>
       <c r="B35" t="str">
-        <v>사람들과 함께할 때 내가 중심이 되어, 내가 생각한 방향대로 상황을 풀어나가려는 편이다.</v>
+        <v>여러 사람이 함께 할 때 분위기를 주도하며, 내 뜻대로 상황을 이끌어가곤 한다.</v>
       </c>
       <c r="C35" t="str">
         <v>cp_negative</v>
@@ -1006,7 +1006,7 @@
         <v>35</v>
       </c>
       <c r="B36" t="str">
-        <v>누구나 실수를 통해 배우며, 더 나은 사람으로 성장할 잠재력이 있다고 믿는다.</v>
+        <v>사람마다 각자의 생각과 의견을, 자유롭게 갖는 것은 당연하며 존중한다.</v>
       </c>
       <c r="C36" t="str">
         <v>u_plus</v>
@@ -1023,7 +1023,7 @@
         <v>36</v>
       </c>
       <c r="B37" t="str">
-        <v>마음속에 불만이나 서운함이 쌓여도, 겉으로 솔직하게 말하지 못하고 속으로 삭이는 편이다.</v>
+        <v>마음속에 불만이나 서운함이 생겨도, 겉으로 내색하지 않고 속으로 참아내곤 한다.</v>
       </c>
       <c r="C37" t="str">
         <v>ac_negative</v>
@@ -1040,7 +1040,7 @@
         <v>37</v>
       </c>
       <c r="B38" t="str">
-        <v>어떤 일이든 망설이지 않고, 스스로 상황을 이끌며 적극적으로 행동하는 편이다.</v>
+        <v>어떤 일이 주어지든, 스스로를 믿고 일을 잘 이끌어가려는 편이다.</v>
       </c>
       <c r="C38" t="str">
         <v>i_plus</v>
@@ -1074,7 +1074,7 @@
         <v>39</v>
       </c>
       <c r="B40" t="str">
-        <v>갈등이나 문제가 생기면 원인을 따져보기도 전에, 무조건 내 잘못으로 생긴 일이라고 생각하는 편이다.</v>
+        <v>스스로 결정하는 게 불안해서, 주로 다른 사람의 의견을 더 따르는 편이다.</v>
       </c>
       <c r="C40" t="str">
         <v>i_minus</v>
@@ -1091,7 +1091,7 @@
         <v>40</v>
       </c>
       <c r="B41" t="str">
-        <v>다른 사람의 주장이나 의견을 들으면, 솔직히 깊이가 없거나 틀렸다는 생각이 먼저 드는 편이다.</v>
+        <v>상대 방식이 내 기대와 다르면, 쉽게 마음에 걸리는 편이다.</v>
       </c>
       <c r="C41" t="str">
         <v>u_minus</v>
@@ -1108,7 +1108,7 @@
         <v>41</v>
       </c>
       <c r="B42" t="str">
-        <v>사람들과 함께할 때 서로 호흡을 맞추며, 손발을 잘 맞추어 나가는 편이다.</v>
+        <v>사람들과 함께 일하거나 활동할 때, 호흡을 맞추며 조화롭게 협조하는 편이다.</v>
       </c>
       <c r="C42" t="str">
         <v>ac_positive</v>
@@ -1125,7 +1125,7 @@
         <v>42</v>
       </c>
       <c r="B43" t="str">
-        <v>어떤 일이나 관계를 맺을 때, 나에게 돌아올 득과 실을 먼저 계산해보는 편이다.</v>
+        <v>어떤 일을 시작할 때, 실질적으로 이득이 되는지 먼저 살펴보곤 한다.</v>
       </c>
       <c r="C43" t="str">
         <v>a_negative</v>
@@ -1142,7 +1142,7 @@
         <v>43</v>
       </c>
       <c r="B44" t="str">
-        <v>상대방의 이야기를 귀담아듣고, 그 마음을 깊이 헤아리며 받아주고자 노력하는 편이다.</v>
+        <v>다른 사람을 마음 깊이 배려하고, 따뜻하게 보살펴 주곤 한다.</v>
       </c>
       <c r="C44" t="str">
         <v>np_positive</v>
@@ -1159,7 +1159,7 @@
         <v>44</v>
       </c>
       <c r="B45" t="str">
-        <v>공공의 규칙과 질서를 대체로 잘 지키며, 원칙에 맞게 바르게 행동하려 노력하는 편이다.</v>
+        <v>눈앞의 작은 이익에 흔들리지 않고, 양심과 올바른 기준에 따라 행동하곤 한다.</v>
       </c>
       <c r="C45" t="str">
         <v>cp_positive</v>
@@ -1176,7 +1176,7 @@
         <v>45</v>
       </c>
       <c r="B46" t="str">
-        <v>남들의 기준과 상관없이, 내 외모에는 나만의 고유한 매력과 개성이 있다고 느낀다.</v>
+        <v>스스로의 외모나 인상에 대해 나름대로 만족하는 편이다.</v>
       </c>
       <c r="C46" t="str">
         <v>i_plus</v>
@@ -1193,7 +1193,7 @@
         <v>46</v>
       </c>
       <c r="B47" t="str">
-        <v>차분히 생각하기보다, 순간의 충동에 이끌려 즉흥적으로 행동하곤 한다.</v>
+        <v>깊이 따져보기보다, 순간의 흥미나 호기심에 끌려 섣불리 결정해 버리곤 한다.</v>
       </c>
       <c r="C47" t="str">
         <v>fc_negative</v>
@@ -1210,7 +1210,7 @@
         <v>47</v>
       </c>
       <c r="B48" t="str">
-        <v>동료나 주변 사람이 실수를 하더라도, 비난하기보다 따뜻하게 격려하고 지지해 주는 편이다.</v>
+        <v>동료가 실수나 실패를 하더라도, 비난하지 않고 따뜻하게 격려하는 편이다.</v>
       </c>
       <c r="C48" t="str">
         <v>u_plus</v>
@@ -1244,7 +1244,7 @@
         <v>49</v>
       </c>
       <c r="B50" t="str">
-        <v>마음이 힘들거나 지칠 때면, 내가 아무런 쓸모가 없는 사람이라 생각하는 편이다.</v>
+        <v>마음이 지치고 힘들 때면, 나 자신이 별로 가치 없게 느껴지기도 한다.</v>
       </c>
       <c r="C50" t="str">
         <v>i_minus</v>
@@ -1261,7 +1261,7 @@
         <v>50</v>
       </c>
       <c r="B51" t="str">
-        <v>다른 사람이 한 일이 내 마음에 들지 않으면, 쉽게 짜증이 나거나 화가 나는 편이다.</v>
+        <v>내가 맡긴 일이 기대에 미치지 못하면, 상대의 시정보다 잘못된 점을 먼저 따지는 편이다.</v>
       </c>
       <c r="C51" t="str">
         <v>u_minus</v>
@@ -1278,7 +1278,7 @@
         <v>51</v>
       </c>
       <c r="B52" t="str">
-        <v>막연한 생각이나 감정에 사로잡히지 않고, 현실적이고 이성적으로 판단하는 편이다.</v>
+        <v>막연한 기대에 이끌리기보다, 현재 상황을 있는 그대로 직시하며 대응하곤 한다.</v>
       </c>
       <c r="C52" t="str">
         <v>a_positive</v>
@@ -1295,7 +1295,7 @@
         <v>52</v>
       </c>
       <c r="B53" t="str">
-        <v>다른 사람의 사소한 일이나 문제까지도, 지나치게 걱정하고 마음을 졸이는 편이다.</v>
+        <v>다른 사람이 개인적인 문제나 사정까지 깊이 신경 쓰곤 한다.</v>
       </c>
       <c r="C53" t="str">
         <v>np_negative</v>
@@ -1312,7 +1312,7 @@
         <v>53</v>
       </c>
       <c r="B54" t="str">
-        <v>복잡하게 생각하기보다 직감이나 감각으로, 상황을 빠르게 파악해 내는 편이다.</v>
+        <v>복잡하게 따지기보다, 직관이나 감각을 활용해 상황을 빠르게 파악하곤 한다.</v>
       </c>
       <c r="C54" t="str">
         <v>fc_positive</v>
@@ -1329,7 +1329,7 @@
         <v>54</v>
       </c>
       <c r="B55" t="str">
-        <v>내 생각과 방식이 옳다는 확신이 강해서, 다른 사람도 내 기준을 따르기를 바라는 편이다.</v>
+        <v>상식이나 기준에 맞지 않는 행동을 보면, 이해가 되지 않고 대체로 거부감이 든다.</v>
       </c>
       <c r="C55" t="str">
         <v>cp_negative</v>
@@ -1346,7 +1346,7 @@
         <v>55</v>
       </c>
       <c r="B56" t="str">
-        <v>어릴 때부터 주변의 따뜻한 보살핌과 사랑을 받으며 자란 편이다.</v>
+        <v>어릴 적 주변의 사랑과 보살핌 속에서 자연스럽게 자라왔다고 생각한다.</v>
       </c>
       <c r="C56" t="str">
         <v>i_plus</v>
@@ -1363,7 +1363,7 @@
         <v>56</v>
       </c>
       <c r="B57" t="str">
-        <v>사소한 일도 스스로 결정을 내리지 못하고 망설이다가, 대체로 남의 의견에 따르곤 한다.</v>
+        <v>사소한 선택도 혼자 내리지 못해 주저하다가, 결국 남들이 하자고 하는 대로 따르곤 한다.</v>
       </c>
       <c r="C57" t="str">
         <v>ac_negative</v>
@@ -1380,7 +1380,7 @@
         <v>57</v>
       </c>
       <c r="B58" t="str">
-        <v>다른 사람의 단점이나 부족한 점도, 있는 그대로 편견 없이 받아들이는 편이다.</v>
+        <v>상대의 기분이나 상황을 헤아리려, 노력하는 편이다.</v>
       </c>
       <c r="C58" t="str">
         <v>u_plus</v>
@@ -1414,7 +1414,7 @@
         <v>59</v>
       </c>
       <c r="B60" t="str">
-        <v>잘못되거나 실패할까 봐 불안해서, 새로운 일에 나서는 것을 주저하는 편이다.</v>
+        <v>혹시나 실수하거나 망신을 당할까 봐, 새로운 일에 선뜻 도전하지 못하는 편이다.</v>
       </c>
       <c r="C60" t="str">
         <v>i_minus</v>
@@ -1431,7 +1431,7 @@
         <v>60</v>
       </c>
       <c r="B61" t="str">
-        <v>나와 생각이나 가치관이 다른 사람을 보면, 이해하기보다 반감이 먼저 드는 편이다.</v>
+        <v>나와 생각이 다른 사람의 의견을 들으면, 내심 잘 받아들여지지 않는 편이다.</v>
       </c>
       <c r="C61" t="str">
         <v>u_minus</v>
@@ -1448,7 +1448,7 @@
         <v>61</v>
       </c>
       <c r="B62" t="str">
-        <v>주변 사람들로부터 예의 바르고 온화하다는 말을 자주 듣는 편이다.</v>
+        <v>주변 사람들로부터 예의 바르고 배려심이 깊다는 이야기를, 자주 듣는 편이다.</v>
       </c>
       <c r="C62" t="str">
         <v>ac_positive</v>
@@ -1465,7 +1465,7 @@
         <v>62</v>
       </c>
       <c r="B63" t="str">
-        <v>사소한 의문이라도 그냥 넘어가지 못하고, 상대에게 끝까지 따져 묻는 편이다.</v>
+        <v>이해가 잘 되지 않거나 의문이 생기면, 끝까지 구체적인 근거를 확인하곤 한다.</v>
       </c>
       <c r="C63" t="str">
         <v>a_negative</v>
@@ -1482,7 +1482,7 @@
         <v>63</v>
       </c>
       <c r="B64" t="str">
-        <v>주변 사람들이나 후배들을 따뜻하게 챙기고, 잘 성장하도록 힘이 되어주려 하는 편이다.</v>
+        <v>후배나 동료들이 잘 성장할 수 있게, 따뜻하게 품어 힘이 되어주곤 한다.</v>
       </c>
       <c r="C64" t="str">
         <v>np_positive</v>
@@ -1499,7 +1499,7 @@
         <v>64</v>
       </c>
       <c r="B65" t="str">
-        <v>옳은 일이라고 판단되면, 주저 없이 앞장서서 이끌곤 한다.</v>
+        <v>옳다고 생각하는 일에는 주저하지 않고, 소신 있게 소리를 내거나 행동하곤 한다.</v>
       </c>
       <c r="C65" t="str">
         <v>cp_positive</v>
@@ -1516,7 +1516,7 @@
         <v>65</v>
       </c>
       <c r="B66" t="str">
-        <v>완벽하진 않더라도, 나만의 강점과 능력에는 솔직히 자신감이 있는 편이다.</v>
+        <v>나에게도 특정한 분야나 능력에서는 확실히 자신감이 있는 편이다.</v>
       </c>
       <c r="C66" t="str">
         <v>i_plus</v>
@@ -1533,7 +1533,7 @@
         <v>66</v>
       </c>
       <c r="B67" t="str">
-        <v>작은 흥미에도 쉽게 일을 시작하지만, 마무리는 대체로 흐지부지되는 편이다.</v>
+        <v>상황이나 상대의 기분을 세심히 살피기보다는, 내 감정을 솔직하게 드러내곤 한다.</v>
       </c>
       <c r="C67" t="str">
         <v>fc_negative</v>
@@ -1550,7 +1550,7 @@
         <v>67</v>
       </c>
       <c r="B68" t="str">
-        <v>사람들은 기본적으로 따뜻한 마음과 양심을 가지고 있다고 믿는 편이다.</v>
+        <v>다른 사람을 쉽게 의심하기보다는, 대체로 신뢰하는 편이다.</v>
       </c>
       <c r="C68" t="str">
         <v>u_plus</v>
@@ -1584,7 +1584,7 @@
         <v>69</v>
       </c>
       <c r="B70" t="str">
-        <v>남들은 신경 쓰지도 않을 사소한 말이나 행동을, 혼자 끊임없이 되짚어보며 괴로워하는 편이다.</v>
+        <v>지나간 사소한 언행이나 행동이 마음에 걸려, 속으로 자주 후회하는 편이다.</v>
       </c>
       <c r="C70" t="str">
         <v>i_minus</v>
@@ -1601,7 +1601,7 @@
         <v>70</v>
       </c>
       <c r="B71" t="str">
-        <v>누군가를 대할 때, 그 사람의 장점보다 단점이나 아쉬운 점이 먼저 보이는 편이다.</v>
+        <v>사람들을 대할 때 긍정적인 면보다는, 아쉬운 점이나 단점이 먼저 보이는 편이다.</v>
       </c>
       <c r="C71" t="str">
         <v>u_minus</v>
@@ -1618,7 +1618,7 @@
         <v>71</v>
       </c>
       <c r="B72" t="str">
-        <v>일을 시작할 때 즉흥적으로 나서기보다, 구체적인 계획을 세워 차근차근 실행하는 편이다.</v>
+        <v>중요한 일을 추진할 때 사전에 계획을 세우고, 순서대로 차근차근 진행하는 편이다.</v>
       </c>
       <c r="C72" t="str">
         <v>a_positive</v>
@@ -1635,7 +1635,7 @@
         <v>72</v>
       </c>
       <c r="B73" t="str">
-        <v>다른 사람이 부탁하지 않았는데도, 나서서 챙겨주거나 관여하는 편이다.</v>
+        <v>남이 따로 요청하지 않아도, 먼저 나서서 일을 대신 해결해 주곤 한다.</v>
       </c>
       <c r="C73" t="str">
         <v>np_negative</v>
@@ -1652,7 +1652,7 @@
         <v>73</v>
       </c>
       <c r="B74" t="str">
-        <v>평소 활기차게 생활하며, 밝고 긍정적인 편이다.</v>
+        <v>시끌벅적 즐겁게 어울릴 때, 때로 구속받지 않고 발랄한 태도로 행동하곤 한다.</v>
       </c>
       <c r="C74" t="str">
         <v>fc_positive</v>
@@ -1669,7 +1669,7 @@
         <v>74</v>
       </c>
       <c r="B75" t="str">
-        <v>다른 사람의 말이나 행동에 대해, 나도 모르게 비판적인 시선으로 엄격하게 평가하곤 한다.</v>
+        <v>상황이 뜻대로 되지 않으면, 나도 모르게 불만이나 날카로움을 표현하곤 한다.</v>
       </c>
       <c r="C75" t="str">
         <v>cp_negative</v>
@@ -1686,7 +1686,7 @@
         <v>75</v>
       </c>
       <c r="B76" t="str">
-        <v>다른 사람들이 해내는 일이라면, 나도 노력하면 충분히 해낼 수 있다고 믿는 편이다.</v>
+        <v>다른 사람들이 해내는 평범한 일 정도는, 나도 충분히 해낼 수 있다고 생각한다.</v>
       </c>
       <c r="C76" t="str">
         <v>i_plus</v>
@@ -1703,7 +1703,7 @@
         <v>76</v>
       </c>
       <c r="B77" t="str">
-        <v>부담스러운 부탁을 받아도, 상대방이 실망하거나 싫어할까 봐 단호하게 거절하지 못하곤 한다.</v>
+        <v>내키지 않거나 부담스러운 부탁을 받아도, 거절하지 못하고 난감해하곤 한다.</v>
       </c>
       <c r="C77" t="str">
         <v>ac_negative</v>
@@ -1720,7 +1720,7 @@
         <v>77</v>
       </c>
       <c r="B78" t="str">
-        <v>사람들과 편안하게 마음을 나누다 보면, 함께하는 것만으로도 큰 힘과 활력을 얻는 편이다.</v>
+        <v>주변 사람들과 대체로 좋은 관계를 이어가는 편이다.</v>
       </c>
       <c r="C78" t="str">
         <v>u_plus</v>
@@ -1754,7 +1754,7 @@
         <v>79</v>
       </c>
       <c r="B80" t="str">
-        <v>다른 사람과 나를 비교하다 보면, 내가 뒤처지고 초라하게 느껴지곤 한다.</v>
+        <v>사람들과 어울리는 게 살짝 부담스러워, 혼자 시간을 보내는 것을 더 선호하는 편이다.</v>
       </c>
       <c r="C80" t="str">
         <v>i_minus</v>
@@ -1771,7 +1771,7 @@
         <v>80</v>
       </c>
       <c r="B81" t="str">
-        <v>사람들은 대개 이기적이고 계산적이어서, 온전히 믿기는 어렵다고 생각하는 편이다.</v>
+        <v>약속이나 형식을 지키지 않으면, 불편하게 느끼는 편이다.</v>
       </c>
       <c r="C81" t="str">
         <v>u_minus</v>
@@ -1788,7 +1788,7 @@
         <v>81</v>
       </c>
       <c r="B82" t="str">
-        <v>갈등을 만들기보다 다른 사람의 의견을 존중하며, 유연하게 맞춰가는 편이다.</v>
+        <v>대인관계에서 내 고집만 피우기보다, 타인의 의견을 유연하게 받아들이곤 한다.</v>
       </c>
       <c r="C82" t="str">
         <v>ac_positive</v>
@@ -1805,7 +1805,7 @@
         <v>82</v>
       </c>
       <c r="B83" t="str">
-        <v>대체로 원칙과 효율에만 얽매여, 융통성과 인간미가 부족하다는 말을 듣곤 한다.</v>
+        <v>상황의 가변성보다, 정해진 기준과 수치에 따라 정확히 일하려고 한다.</v>
       </c>
       <c r="C83" t="str">
         <v>a_negative</v>
@@ -1822,7 +1822,7 @@
         <v>83</v>
       </c>
       <c r="B84" t="str">
-        <v>다른 사람이 실수하더라도 다그치기보다, 너그럽게 감싸주고 이해하려는 편이다.</v>
+        <v>타인의 실수를 나무라기보다, 너그럽게 이해하고 받아들이곤 한다.</v>
       </c>
       <c r="C84" t="str">
         <v>np_positive</v>
@@ -1839,7 +1839,7 @@
         <v>84</v>
       </c>
       <c r="B85" t="str">
-        <v>현재의 편안함과 타협하지 않고, 가치 있는 꿈과 높은 이상을 향해 노력하는 편이다.</v>
+        <v>어디에서나 공공질서와 기본 예의를, 대체로 잘 지키고 있다.</v>
       </c>
       <c r="C85" t="str">
         <v>cp_positive</v>
@@ -1856,7 +1856,7 @@
         <v>85</v>
       </c>
       <c r="B86" t="str">
-        <v>사람들 앞에서는 대체로 긴장하지 않고, 내 생각을 자연스럽고 당당하게 표현하는 편이다.</v>
+        <v>사람들 앞에서 위축되기보다, 내 생각이나 마음을 편안하게 표현하려는 편이다.</v>
       </c>
       <c r="C86" t="str">
         <v>i_plus</v>
@@ -1873,7 +1873,7 @@
         <v>86</v>
       </c>
       <c r="B87" t="str">
-        <v>조심스럽고 진지해야 할 자리에서도 나도 모르게, 가볍거나 장난스럽게 행동하곤 한다.</v>
+        <v>조심스럽고 진지해야 할 자리에서 나도 모르게, 가볍거나 장난스럽게 행동하곤 한다.</v>
       </c>
       <c r="C87" t="str">
         <v>fc_negative</v>
@@ -1890,7 +1890,7 @@
         <v>87</v>
       </c>
       <c r="B88" t="str">
-        <v>모든 사람은 각자의 생각과 감정을 존중받아야 할, 소중한 존재라고 여긴다.</v>
+        <v>누구나 스스로 판단하고 결정하는 것은, 당연한 권리라고 생각한다.</v>
       </c>
       <c r="C88" t="str">
         <v>u_plus</v>
@@ -1924,7 +1924,7 @@
         <v>89</v>
       </c>
       <c r="B90" t="str">
-        <v>스스로 내세울 점이 별로 없다고 느껴져, 늘 자신이 없고 위축되는 편이다.</v>
+        <v>스스로 내세울 점이 별로 없다고 느껴져, 늘 자신감이 떨어지는 편이다.</v>
       </c>
       <c r="C90" t="str">
         <v>i_minus</v>
@@ -1941,7 +1941,7 @@
         <v>90</v>
       </c>
       <c r="B91" t="str">
-        <v>남에게 온전히 맡기기가 불안해서, 중요한 일일수록 내가 직접 챙기는 편이다.</v>
+        <v>남에게 일을 믿고 맡기기보다는, 내가 직접 처리하려는 편이다.</v>
       </c>
       <c r="C91" t="str">
         <v>u_minus</v>
@@ -1958,7 +1958,7 @@
         <v>91</v>
       </c>
       <c r="B92" t="str">
-        <v>대체로 감정에 치우치기보다, 상황을 객관적이고 합리적으로 판단하여 일을 처리하는 편이다.</v>
+        <v>복잡한 문제가 생겨도 감정적으로 굴지 않고, 차분히 합리적인 해결책을 찾으려 한다.</v>
       </c>
       <c r="C92" t="str">
         <v>a_positive</v>
@@ -1975,7 +1975,7 @@
         <v>92</v>
       </c>
       <c r="B93" t="str">
-        <v>상대가 딱해 보이면 마음이 약해져서, 조금 무리가 되더라도 부탁을 들어주곤 한다.</v>
+        <v>상대방의 사정이 딱하게 느껴지면, 무리가 되더라도 부탁을 들어주곤 한다.</v>
       </c>
       <c r="C93" t="str">
         <v>np_negative</v>
@@ -1992,7 +1992,7 @@
         <v>93</v>
       </c>
       <c r="B94" t="str">
-        <v>상대방에게 화가 나면 감정을 다스리지 못하고, 거친 말을 쏟아붓는 편이다.</v>
+        <v>상대방이 잘못을 했을 때, 때로는 심하게 몰아붙이거나 비난할 때도 있다.</v>
       </c>
       <c r="C94" t="str">
         <v>u_minus</v>
@@ -2009,7 +2009,7 @@
         <v>94</v>
       </c>
       <c r="B95" t="str">
-        <v>내가 속한 모임이나 조직의 방침 안에서, 튀지 않고 성실하게 행동하는 편이다.</v>
+        <v>나 혼자 독단적으로 결정하기보다, 주변 상황과 의견에 맞추어 행동하는 편이다.</v>
       </c>
       <c r="C95" t="str">
         <v>ac_positive</v>
@@ -2026,7 +2026,7 @@
         <v>95</v>
       </c>
       <c r="B96" t="str">
-        <v>나에게 맡겨진 일에 대해서는, 끝까지 책임을 다해 마무리하는 편이다.</v>
+        <v>나에게 맡겨진 일이 다소 힘들더라도, 책임감을 가지고 끝까지 해내곤 한다.</v>
       </c>
       <c r="C96" t="str">
         <v>cp_positive</v>
@@ -2043,7 +2043,7 @@
         <v>96</v>
       </c>
       <c r="B97" t="str">
-        <v>누구를 만나더라도 그 사람의 장점이나 배울 점을 먼저 보려는 편이다.</v>
+        <v>마음에 들지 않는 사람과도, 과업을 위해서라면 함께 일하는 편이다.</v>
       </c>
       <c r="C97" t="str">
         <v>u_plus</v>
@@ -2060,7 +2060,7 @@
         <v>97</v>
       </c>
       <c r="B98" t="str">
-        <v>내가 내린 판단과 결정을 확신하기 어려워, 일을 처리하는 동안 자주 불안감을 느끼는 편이다.</v>
+        <v>혼자 결정하는 게 부담스러워서, 쉽게 결단을 내리지 못하는 편이다.</v>
       </c>
       <c r="C98" t="str">
         <v>i_minus</v>
@@ -2077,7 +2077,7 @@
         <v>98</v>
       </c>
       <c r="B99" t="str">
-        <v>일이 잘 풀리지 않더라도 금방 낙담하지 않고, 다시 시도해 보려는 편이다.</v>
+        <v>일이 뜻대로 잘 풀리지 않더라도 쉽게 포기하지 않고, 다시 시도해 보려는 편이다.</v>
       </c>
       <c r="C99" t="str">
         <v>i_plus</v>
@@ -2094,7 +2094,7 @@
         <v>99</v>
       </c>
       <c r="B100" t="str">
-        <v>호기심과 상상력이 풍부해서, 엉뚱하거나 새로운 아이디어를 잘 떠올리는 편이다.</v>
+        <v>풍부한 상상력을 바탕으로, 가끔 참신한 아이디어를 잘 떠올리곤 한다.</v>
       </c>
       <c r="C100" t="str">
         <v>fc_positive</v>

</xml_diff>